<commit_message>
docs(proposal): v1.6.1 — AI internal engineering ditetapkan Claude Max $200/bln
Keputusan founder/CTO: tier Claude Code Max $200/bln (dari asumsi $100).
Dampak dihitung ulang menyeluruh: software Launch ~5,1 jt/bln; PLAFON
12 bln Rp 85 jt -> Rp 105 jt (realisasi ~97 jt = 51% alokasi PRD 2027;
skenario dini ~103 jt); fase Launch ~5,9 jt/bln, Growth ~8,5 jt/bln,
Scale ~21 jt/bln; plot 3 th ~Rp 855 jt = 104% alokasi PRD — disclosure
jujur: perlu revisi minor alokasi PRD 14.4 atau ditutup dari pos lain
(keputusan stakeholder). A15 dikunci; Excel AIENG=200 + plafon + label;
ringkasan-pengajuan + tabel gabungan SDM diselaraskan; changelog v1.6.1.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AdopTreeWorld/proposal/perhitungan-kapasitas-anggaran-adoptree.xlsx
+++ b/AdopTreeWorld/proposal/perhitungan-kapasitas-anggaran-adoptree.xlsx
@@ -64,13 +64,13 @@
     <t>Anggaran 12 bulan pertama (Agu 2026 – Jul 2027)</t>
   </si>
   <si>
-    <t>Total proyeksi realisasi — base, upgrade per trigger (termasuk buffer 10%); skenario upgrade dini ≈ Rp 82 jt di sheet Anggaran12Bln (v1.6: termasuk ArcGIS + AccuWeather + AI)</t>
+    <t>Total proyeksi realisasi — base, upgrade per trigger (termasuk buffer 10%); skenario upgrade dini ≈ Rp 103 jt di sheet Anggaran12Bln (v1.6.1: termasuk ArcGIS + AccuWeather + Claude Max $200)</t>
   </si>
   <si>
     <t>PLAFON diajukan untuk persetujuan</t>
   </si>
   <si>
-    <t>Rasio realisasi base terhadap alokasi infrastruktur PRD §14.4 tahun 2027 (plafon ≈ 45%)</t>
+    <t>Rasio realisasi base terhadap alokasi infrastruktur PRD §14.4 tahun 2027 (plafon ≈ 55%)</t>
   </si>
   <si>
     <t>Cara pakai: seluruh sel KUNING di sheet Asumsi adalah input — ubah nilainya (kurs, %DAU, harga, volume anchor) dan seluruh workbook menghitung ulang.</t>
@@ -448,7 +448,7 @@
     <t>AIENG</t>
   </si>
   <si>
-    <t>AI internal engineering per bulan (USD; Claude/GPT, 1 seat Pro→Max)</t>
+    <t>AI internal engineering per bulan (USD; Claude Code Max $200 — rekomendasi CTO, 1 seat)</t>
   </si>
   <si>
     <t>Model Beban — formula eksplisit dari anchor PRD §14.2 (dokumen §3)</t>
@@ -943,7 +943,7 @@
     <t>menampung base maupun skenario upgrade dini (baris 22–25)</t>
   </si>
   <si>
-    <t>85000000</t>
+    <t>105000000</t>
   </si>
   <si>
     <t>Ruang tersisa terhadap plafon</t>
@@ -3624,13 +3624,13 @@
         <v>142</v>
       </c>
       <c r="C45" s="16">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="D45" s="16">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E45" s="16">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(proposal): Excel selaras penuh v1.6.1 — sheet OnPremise + label Claude Max
Audit menyeluruh workbook: sheet OnPremise dikoreksi — catatan realisasi
Th-1 (40 jt -> 97 jt), formula Th-3 & Th-4+ kini menambahkan langganan
strategis (Software!E22:E24) yang tetap berjalan pasca-cutover on-premise
(sebelumnya hanya OpEx+amortisasi), catatan total 3 th ~855 jt (104%
alokasi, rujuk disclosure 10.5). Label AI internal di Software & Asumsi
dikunci "Claude Code Max $200/bln (rekomendasi CTO)". Sheet lain sudah
formula-driven dan otomatis mengikuti (Ringkasan/Anggaran12Bln/Server).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AdopTreeWorld/proposal/perhitungan-kapasitas-anggaran-adoptree.xlsx
+++ b/AdopTreeWorld/proposal/perhitungan-kapasitas-anggaran-adoptree.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="490">
   <si>
     <t>AdopTree World — Perhitungan Kapasitas &amp; Anggaran Infrastruktur (Staging + Production)</t>
   </si>
@@ -808,7 +808,7 @@
     <t>Trial gratis → Standard $25 (225 rb calls) → Elite $500</t>
   </si>
   <si>
-    <t>AI internal engineering — Claude Code / ChatGPT</t>
+    <t>AI internal engineering — Claude Code Max $200/bln (rekomendasi CTO)</t>
   </si>
   <si>
     <t>AIENG × KURS</t>
@@ -1234,7 +1234,7 @@
     <t>Cloud — plafon proposal ini</t>
   </si>
   <si>
-    <t>realisasi ≈ Rp 40 jt</t>
+    <t>realisasi ≈ Rp 97 jt (v1.6.1 — termasuk langganan strategis)</t>
   </si>
   <si>
     <t>Tahun 2 (Agu 2027–Jul 2028)</t>
@@ -1252,7 +1252,7 @@
     <t>Cloud ±8 bln + CapEx on-prem + parallel run 4 bln</t>
   </si>
   <si>
-    <t>cutover bertahap</t>
+    <t>cutover bertahap; 4 bln parallel-run termasuk langganan strategis yang tetap berjalan</t>
   </si>
   <si>
     <t>TOTAL 3 TAHUN</t>
@@ -1261,13 +1261,16 @@
     <t>jumlah</t>
   </si>
   <si>
+    <t>≈ Rp 855 jt (v1.6.1) — ≈104% alokasi PRD: lihat disclosure §10.5 dokumen</t>
+  </si>
+  <si>
     <t>Tahun 4+ (steady on-premise)</t>
   </si>
   <si>
     <t>OpEx + amortisasi × 12</t>
   </si>
   <si>
-    <t>vs tetap cloud &gt; Rp 240–300 jt/th → hemat mulai th-4</t>
+    <t>termasuk langganan strategis (Software!E22:E24) yang tetap berjalan on-premise; vs tetap cloud &gt; Rp 320–380 jt/th → hemat mulai th-4</t>
   </si>
   <si>
     <t>Alokasi infra PRD §14.4 tiga tahun</t>
@@ -2192,22 +2195,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B5" s="16">
         <v>1.2</v>
@@ -2215,7 +2218,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B6" s="16">
         <v>10</v>
@@ -2223,7 +2226,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B7" s="16">
         <v>20</v>
@@ -2231,7 +2234,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B8" s="16">
         <v>3</v>
@@ -2239,7 +2242,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B9" s="16">
         <v>16000</v>
@@ -2247,7 +2250,7 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -2255,39 +2258,39 @@
         <v>20</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="H12" s="38" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="J12" s="38" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B13" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C13" s="39">
         <v>14</v>
@@ -2316,10 +2319,10 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B14" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C14" s="39">
         <v>7</v>
@@ -2348,10 +2351,10 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B15" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C15" s="39">
         <v>8</v>
@@ -2380,10 +2383,10 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B16" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C16" s="39">
         <v>9</v>
@@ -2412,10 +2415,10 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B17" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C17" s="39">
         <v>15</v>
@@ -2444,10 +2447,10 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B18" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C18" s="39">
         <v>14</v>
@@ -2476,10 +2479,10 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B19" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C19" s="39">
         <v>6.5</v>
@@ -2508,10 +2511,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B20" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C20" s="39">
         <v>8</v>
@@ -2540,10 +2543,10 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B21" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C21" s="39">
         <v>7</v>
@@ -2572,10 +2575,10 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B22" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C22" s="39">
         <v>15</v>
@@ -2604,10 +2607,10 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B23" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C23" s="39">
         <v>16</v>
@@ -2636,10 +2639,10 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B24" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C24" s="39">
         <v>10</v>
@@ -2668,10 +2671,10 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B25" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C25" s="39">
         <v>12</v>
@@ -2700,10 +2703,10 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B26" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C26" s="39">
         <v>16</v>
@@ -2732,10 +2735,10 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B27" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D27">
         <v>3</v>
@@ -2763,7 +2766,7 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="H29" s="21"/>
       <c r="I29" s="21"/>
@@ -2771,7 +2774,7 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
@@ -2791,7 +2794,7 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
@@ -2811,24 +2814,24 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B34" s="17">
         <f>5*H31</f>
       </c>
       <c r="D34" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E34" s="17">
         <f>36000*$B$9/1000000</f>
       </c>
       <c r="F34" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="G34" s="40">
         <f>B34/E34</f>
@@ -2836,19 +2839,19 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B35" s="17">
         <f>3*(H31+G17+G18)+3*(H31+G17+G18+G19+G15+G20)+6*I31</f>
       </c>
       <c r="D35" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E35" s="17">
         <f>120000*$B$9/1000000</f>
       </c>
       <c r="F35" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="G35" s="40">
         <f>B35/E35</f>
@@ -2856,19 +2859,19 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B36" s="17">
         <f>12*J31</f>
       </c>
       <c r="D36" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E36" s="17">
         <f>360000*$B$9/1000000</f>
       </c>
       <c r="F36" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="G36" s="40">
         <f>B36/E36</f>
@@ -2876,19 +2879,19 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B37" s="17">
         <f>B34+B35+B36</f>
       </c>
       <c r="D37" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E37" s="17">
         <f>E34+E35+E36</f>
       </c>
       <c r="F37" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="G37" s="40">
         <f>B37/E37</f>
@@ -2896,12 +2899,12 @@
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B40" s="17">
         <f>5*H31+3*(H31+G17+G18)+3*(H31+G17+G18+G19+G15+G20)+1*I31</f>
@@ -2909,13 +2912,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B41" s="41">
         <v>1500</v>
       </c>
       <c r="D41" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E41" s="40">
         <f>B40/B41</f>
@@ -2923,23 +2926,23 @@
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="15" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B45">
         <f>0.5*G17</f>
       </c>
       <c r="C45" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
   </sheetData>
@@ -5408,7 +5411,7 @@
         <v>409</v>
       </c>
       <c r="C29" s="4">
-        <f>(8*Ringkasan!E7+C8+4*C16)*(1+Asumsi!$C$19)</f>
+        <f>(8*Ringkasan!E7+C8+4*(C16+SUM(Software!E22:E24)))*(1+Asumsi!$C$19)</f>
       </c>
       <c r="D29" t="s">
         <v>410</v>
@@ -5424,28 +5427,30 @@
       <c r="C30" s="8">
         <f>SUM(C27:C29)</f>
       </c>
-      <c r="D30" s="7"/>
+      <c r="D30" s="7" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B31" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C31" s="4">
-        <f>(C16+C10)*12</f>
+        <f>(C16+C10+SUM(Software!E22:E24))*12</f>
       </c>
       <c r="D31" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B32" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C32" s="4">
         <f>(3600+12000+36000)*Asumsi!$C$4</f>
@@ -5453,10 +5458,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B33" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C33" s="9">
         <f>C30/C32</f>

</xml_diff>

<commit_message>
docs(proposal): v1.6.2 — + Google Workspace (temuan telaah: email domain belum dianggarkan)
Email domain tim (support@/privacy@/security@adoptreeworld.com) sudah
tercantum di halaman legal platform tapi belum masuk pembiayaan — masih
Gmail gratis. Ditambahkan: Google Workspace Business Starter $7/user/bln
(tahunan; terverifikasi harga resmi 2026), seat mengikuti roster SDM
(7 -> 14 -> 21) = Rp 0,78 -> 1,57 -> 2,35 jt/bln. Dibedakan eksplisit
dari Resend/SES (transaksional otomatis vs mailbox manusia).

Dampak: PLAFON 12 bln Rp 105 jt -> Rp 125 jt (realisasi ~114 jt = 60%
alokasi 2027); Launch ~6,7 jt/bln; plot 3 th ~Rp 920 jt = 112% alokasi
PRD — disclosure diperbarui (revisi alokasi +$6.000/3 th atau tutup dari
sisa pos Team). Asumsi A16 + Excel (GWS1/GWS2 sel kuning, Software baris
25, subtotal 22-25, OnPremise ikut, plafon). Ringkasan + tabel gabungan
SDM diselaraskan.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AdopTreeWorld/proposal/perhitungan-kapasitas-anggaran-adoptree.xlsx
+++ b/AdopTreeWorld/proposal/perhitungan-kapasitas-anggaran-adoptree.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="497">
   <si>
     <t>AdopTree World — Perhitungan Kapasitas &amp; Anggaran Infrastruktur (Staging + Production)</t>
   </si>
@@ -64,13 +64,13 @@
     <t>Anggaran 12 bulan pertama (Agu 2026 – Jul 2027)</t>
   </si>
   <si>
-    <t>Total proyeksi realisasi — base, upgrade per trigger (termasuk buffer 10%); skenario upgrade dini ≈ Rp 103 jt di sheet Anggaran12Bln (v1.6.1: termasuk ArcGIS + AccuWeather + Claude Max $200)</t>
+    <t>Total proyeksi realisasi — base, upgrade per trigger (termasuk buffer 10%); skenario upgrade dini ≈ Rp 121 jt di sheet Anggaran12Bln (v1.6.2: termasuk ArcGIS + AccuWeather + Claude Max $200 + Google Workspace)</t>
   </si>
   <si>
     <t>PLAFON diajukan untuk persetujuan</t>
   </si>
   <si>
-    <t>Rasio realisasi base terhadap alokasi infrastruktur PRD §14.4 tahun 2027 (plafon ≈ 55%)</t>
+    <t>Rasio realisasi base terhadap alokasi infrastruktur PRD §14.4 tahun 2027 (plafon ≈ 66%)</t>
   </si>
   <si>
     <t>Cara pakai: seluruh sel KUNING di sheet Asumsi adalah input — ubah nilainya (kurs, %DAU, harga, volume anchor) dan seluruh workbook menghitung ulang.</t>
@@ -451,6 +451,18 @@
     <t>AI internal engineering per bulan (USD; Claude Code Max $200 — rekomendasi CTO, 1 seat)</t>
   </si>
   <si>
+    <t>GWS1</t>
+  </si>
+  <si>
+    <t>Google Workspace Business Starter per user per bulan (USD; paket tahunan)</t>
+  </si>
+  <si>
+    <t>GWS2</t>
+  </si>
+  <si>
+    <t>Seat Workspace per fase (= headcount roster SDM)</t>
+  </si>
+  <si>
     <t>Model Beban — formula eksplisit dari anchor PRD §14.2 (dokumen §3)</t>
   </si>
   <si>
@@ -763,10 +775,10 @@
     <t>SUBTOTAL SOFTWARE</t>
   </si>
   <si>
-    <t>jumlah baris 4–14 + langganan strategis (baris 22–24)</t>
-  </si>
-  <si>
-    <t>v1.6: termasuk ArcGIS + AccuWeather + AI internal; Tira = DeepSeek</t>
+    <t>jumlah baris 4–14 + langganan strategis (baris 22–25)</t>
+  </si>
+  <si>
+    <t>v1.6.2: termasuk ArcGIS + AccuWeather + AI internal + Google Workspace; Tira = DeepSeek</t>
   </si>
   <si>
     <t>Metrik volume (dasar formula di atas)</t>
@@ -787,7 +799,7 @@
     <t>DAU × EML2 × EML1</t>
   </si>
   <si>
-    <t>Langganan strategis (keputusan founder 18 Jul 2026 — v1.6; masuk SUBTOTAL baris 15)</t>
+    <t>Langganan strategis (keputusan founder 18 Jul 2026 — v1.6.2; masuk SUBTOTAL baris 15, baris 22–25)</t>
   </si>
   <si>
     <t>ArcGIS Online (Esri) — analisis GIS profesional &amp; peta MRV</t>
@@ -817,6 +829,15 @@
     <t>khusus internal engineering (komersial = DeepSeek, baris 7)</t>
   </si>
   <si>
+    <t>Google Workspace — email domain tim + Drive/Docs/Meet (beda dari Resend/SES: ini mailbox manusia)</t>
+  </si>
+  <si>
+    <t>GWS1 × seat × KURS</t>
+  </si>
+  <si>
+    <t>Business Starter $7/user/bln (tahunan); support@/privacy@/security@adoptreeworld.com</t>
+  </si>
+  <si>
     <t>Spesifikasi &amp; Harga Server per Tier (dokumen §5) — rentang = harga pasar 4 provider (sheet Pembanding)</t>
   </si>
   <si>
@@ -943,7 +964,7 @@
     <t>menampung base maupun skenario upgrade dini (baris 22–25)</t>
   </si>
   <si>
-    <t>105000000</t>
+    <t>125000000</t>
   </si>
   <si>
     <t>Ruang tersisa terhadap plafon</t>
@@ -2195,22 +2216,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="B5" s="16">
         <v>1.2</v>
@@ -2218,7 +2239,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="B6" s="16">
         <v>10</v>
@@ -2226,7 +2247,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="B7" s="16">
         <v>20</v>
@@ -2234,7 +2255,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="B8" s="16">
         <v>3</v>
@@ -2242,7 +2263,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="B9" s="16">
         <v>16000</v>
@@ -2250,7 +2271,7 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -2258,39 +2279,39 @@
         <v>20</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="H12" s="38" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="J12" s="38" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="B13" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="C13" s="39">
         <v>14</v>
@@ -2319,10 +2340,10 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="B14" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="C14" s="39">
         <v>7</v>
@@ -2351,10 +2372,10 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="B15" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="C15" s="39">
         <v>8</v>
@@ -2383,10 +2404,10 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="B16" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="C16" s="39">
         <v>9</v>
@@ -2415,10 +2436,10 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="B17" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="C17" s="39">
         <v>15</v>
@@ -2447,10 +2468,10 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="B18" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="C18" s="39">
         <v>14</v>
@@ -2479,10 +2500,10 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="B19" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="C19" s="39">
         <v>6.5</v>
@@ -2511,10 +2532,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="B20" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="C20" s="39">
         <v>8</v>
@@ -2543,10 +2564,10 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="B21" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="C21" s="39">
         <v>7</v>
@@ -2575,10 +2596,10 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="B22" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="C22" s="39">
         <v>15</v>
@@ -2607,10 +2628,10 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="B23" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="C23" s="39">
         <v>16</v>
@@ -2639,10 +2660,10 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="B24" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="C24" s="39">
         <v>10</v>
@@ -2671,10 +2692,10 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="B25" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="C25" s="39">
         <v>12</v>
@@ -2703,10 +2724,10 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="B26" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="C26" s="39">
         <v>16</v>
@@ -2735,10 +2756,10 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="B27" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="D27">
         <v>3</v>
@@ -2766,7 +2787,7 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="H29" s="21"/>
       <c r="I29" s="21"/>
@@ -2774,7 +2795,7 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
@@ -2794,7 +2815,7 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="18" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
@@ -2814,24 +2835,24 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="B34" s="17">
         <f>5*H31</f>
       </c>
       <c r="D34" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="E34" s="17">
         <f>36000*$B$9/1000000</f>
       </c>
       <c r="F34" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="G34" s="40">
         <f>B34/E34</f>
@@ -2839,19 +2860,19 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="B35" s="17">
         <f>3*(H31+G17+G18)+3*(H31+G17+G18+G19+G15+G20)+6*I31</f>
       </c>
       <c r="D35" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="E35" s="17">
         <f>120000*$B$9/1000000</f>
       </c>
       <c r="F35" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="G35" s="40">
         <f>B35/E35</f>
@@ -2859,19 +2880,19 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="B36" s="17">
         <f>12*J31</f>
       </c>
       <c r="D36" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="E36" s="17">
         <f>360000*$B$9/1000000</f>
       </c>
       <c r="F36" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="G36" s="40">
         <f>B36/E36</f>
@@ -2879,19 +2900,19 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="B37" s="17">
         <f>B34+B35+B36</f>
       </c>
       <c r="D37" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
       <c r="E37" s="17">
         <f>E34+E35+E36</f>
       </c>
       <c r="F37" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="G37" s="40">
         <f>B37/E37</f>
@@ -2899,12 +2920,12 @@
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="B40" s="17">
         <f>5*H31+3*(H31+G17+G18)+3*(H31+G17+G18+G19+G15+G20)+1*I31</f>
@@ -2912,13 +2933,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="B41" s="41">
         <v>1500</v>
       </c>
       <c r="D41" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="E41" s="40">
         <f>B40/B41</f>
@@ -2926,23 +2947,23 @@
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="15" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="B45">
         <f>0.5*G17</f>
       </c>
       <c r="C45" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>
@@ -2953,7 +2974,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -3634,6 +3655,40 @@
       </c>
       <c r="E45" s="16">
         <v>200</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>143</v>
+      </c>
+      <c r="B46" t="s">
+        <v>144</v>
+      </c>
+      <c r="C46" s="16">
+        <v>7</v>
+      </c>
+      <c r="D46" s="16">
+        <v>7</v>
+      </c>
+      <c r="E46" s="16">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>145</v>
+      </c>
+      <c r="B47" t="s">
+        <v>146</v>
+      </c>
+      <c r="C47" s="16">
+        <v>7</v>
+      </c>
+      <c r="D47" s="16">
+        <v>14</v>
+      </c>
+      <c r="E47" s="16">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -3655,7 +3710,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -3664,10 +3719,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>116</v>
@@ -3684,7 +3739,7 @@
         <v>120</v>
       </c>
       <c r="B4" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C4" s="17">
         <f>Asumsi!C34</f>
@@ -3698,10 +3753,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C5" s="17">
         <f>C4*Asumsi!$C$5</f>
@@ -3715,10 +3770,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B6" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C6" s="17">
         <f>C5*Asumsi!$C$6</f>
@@ -3732,10 +3787,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B7" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C7" s="17">
         <f>C6*Asumsi!$C$7</f>
@@ -3749,10 +3804,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C8" s="19">
         <f>C7*Asumsi!$C$8</f>
@@ -3766,7 +3821,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -3775,86 +3830,86 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D11" s="18"/>
       <c r="E11" s="18"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B12" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C12" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B13" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C13" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B14" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C14" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B15" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C15" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B16" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C16" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B17" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C17" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3876,7 +3931,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -3885,27 +3940,27 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C4" s="21">
         <f>Asumsi!C35*Asumsi!$C$11*Asumsi!$C$10/1024</f>
@@ -3919,10 +3974,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B5" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C5" s="21">
         <f>Asumsi!C37*Asumsi!$C$13*Asumsi!$C$12/1024</f>
@@ -3936,10 +3991,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B6" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C6" s="21">
         <f>Asumsi!C35*Asumsi!$C$15*Asumsi!$C$14/1024</f>
@@ -3953,10 +4008,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B7" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C7" s="21">
         <f>Asumsi!C36*Asumsi!$C$16</f>
@@ -3970,10 +4025,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B8" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C8" s="21">
         <f>Asumsi!C35*Asumsi!$C$17/1024</f>
@@ -3987,10 +4042,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B9" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C9" s="21">
         <f>Asumsi!C38*117/1024</f>
@@ -4004,10 +4059,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B10" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C10" s="21">
         <f>Asumsi!C39*Asumsi!$C$31</f>
@@ -4021,10 +4076,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C11" s="22">
         <f>SUM(C4:C10)</f>
@@ -4038,10 +4093,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C12" s="22">
         <f>C11*Asumsi!$C$30</f>
@@ -4055,10 +4110,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C13" s="22">
         <f>C11+C12</f>
@@ -4072,10 +4127,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B14" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C14" s="23">
         <f>C13*Asumsi!$C$18</f>
@@ -4089,10 +4144,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B15" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C15" s="24">
         <f>C14*Asumsi!$C$4</f>
@@ -4106,10 +4161,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="20" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B17" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C17" s="25">
         <f>C15*5</f>
@@ -4123,7 +4178,7 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -4134,7 +4189,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -4146,7 +4201,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -4156,30 +4211,30 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C4" s="4">
         <v>0</v>
@@ -4191,15 +4246,15 @@
         <f>20*Asumsi!$C$4</f>
       </c>
       <c r="F4" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B5" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C5" s="4">
         <f>StorageR2!C15</f>
@@ -4216,10 +4271,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B6" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C6" s="4">
         <f>MAX(0,C18-Asumsi!$C$24)/1000*Asumsi!$C$23*Asumsi!$C$4</f>
@@ -4231,15 +4286,15 @@
         <f>MAX(0,E18-Asumsi!$C$24)/1000*Asumsi!$C$23*Asumsi!$C$4</f>
       </c>
       <c r="F6" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B7" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C7" s="4">
         <f>Beban!C5*Asumsi!$C$28*Asumsi!$C$29</f>
@@ -4251,15 +4306,15 @@
         <f>Beban!E5*Asumsi!$C$28*Asumsi!$C$29</f>
       </c>
       <c r="F7" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B8" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C8" s="4">
         <f>IF(C19&lt;=3000,0,IF(C19&lt;=50000,20*Asumsi!$C$4,IF(C19&lt;=100000,90*Asumsi!$C$4,C19/1000*0.1*Asumsi!$C$4)))</f>
@@ -4271,15 +4326,15 @@
         <f>IF(E19&lt;=3000,0,IF(E19&lt;=50000,20*Asumsi!$C$4,IF(E19&lt;=100000,90*Asumsi!$C$4,E19/1000*0.1*Asumsi!$C$4)))</f>
       </c>
       <c r="F8" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B9" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C9" s="4">
         <v>0</v>
@@ -4291,15 +4346,15 @@
         <f>26*Asumsi!$C$4</f>
       </c>
       <c r="F9" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B10" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C10" s="4">
         <v>0</v>
@@ -4313,10 +4368,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B11" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C11" s="4">
         <f>300000/12</f>
@@ -4330,10 +4385,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B12" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C12" s="4">
         <v>0</v>
@@ -4345,15 +4400,15 @@
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B13" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C13" s="4">
         <v>0</v>
@@ -4365,15 +4420,15 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B14" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C14" s="4">
         <v>0</v>
@@ -4385,32 +4440,32 @@
         <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C15" s="27">
-        <f>SUM(C4:C14)+SUM(C22:C24)</f>
+        <f>SUM(C4:C14)+SUM(C22:C25)</f>
       </c>
       <c r="D15" s="27">
-        <f>SUM(D4:D14)+SUM(D22:D24)</f>
+        <f>SUM(D4:D14)+SUM(D22:D25)</f>
       </c>
       <c r="E15" s="27">
-        <f>SUM(E4:E14)+SUM(E22:E24)</f>
+        <f>SUM(E4:E14)+SUM(E22:E25)</f>
       </c>
       <c r="F15" s="26" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6" t="s">
@@ -4426,10 +4481,10 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B18" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C18" s="17">
         <f>Beban!C5*Asumsi!$C$21*Asumsi!$C$22*Asumsi!$C$25</f>
@@ -4441,15 +4496,15 @@
         <f>Beban!E5*Asumsi!$C$21*Asumsi!$C$22*Asumsi!$C$25</f>
       </c>
       <c r="F18" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B19" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="C19" s="17">
         <f>Beban!C5*Asumsi!$C$27*Asumsi!$C$26</f>
@@ -4463,15 +4518,15 @@
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B22" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C22" s="4">
         <f>Asumsi!$C$42*Asumsi!C43*Asumsi!$C$4/12</f>
@@ -4483,15 +4538,15 @@
         <f>Asumsi!$E$42*Asumsi!E43*Asumsi!$C$4/12</f>
       </c>
       <c r="F22" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B23" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C23" s="4">
         <f>Asumsi!C44*Asumsi!$C$4</f>
@@ -4503,15 +4558,15 @@
         <f>Asumsi!E44*Asumsi!$C$4</f>
       </c>
       <c r="F23" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B24" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C24" s="4">
         <f>Asumsi!C45*Asumsi!$C$4</f>
@@ -4523,7 +4578,27 @@
         <f>Asumsi!E45*Asumsi!$C$4</f>
       </c>
       <c r="F24" t="s">
-        <v>264</v>
+        <v>268</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>269</v>
+      </c>
+      <c r="B25" t="s">
+        <v>270</v>
+      </c>
+      <c r="C25" s="4">
+        <f>Asumsi!C46*Asumsi!C47*Asumsi!$C$4</f>
+      </c>
+      <c r="D25" s="4">
+        <f>Asumsi!D46*Asumsi!D47*Asumsi!$C$4</f>
+      </c>
+      <c r="E25" s="4">
+        <f>Asumsi!E46*Asumsi!E47*Asumsi!$C$4</f>
+      </c>
+      <c r="F25" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -4545,7 +4620,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -4554,27 +4629,27 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="B4" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="C4" s="28">
         <v>150000</v>
@@ -4588,10 +4663,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="B5" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="C5" s="28">
         <v>400000</v>
@@ -4605,10 +4680,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B6" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="C6" s="28">
         <v>1300000</v>
@@ -4622,10 +4697,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="B7" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C7" s="28">
         <v>5000000</v>
@@ -4639,10 +4714,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="B8" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="C8" s="28">
         <v>250000</v>
@@ -4656,7 +4731,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="B10" s="29"/>
       <c r="C10" s="29"/>
@@ -4668,12 +4743,12 @@
         <v>2</v>
       </c>
       <c r="B11" s="29" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="C11" s="29"/>
       <c r="D11" s="29"/>
       <c r="E11" s="29" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4681,7 +4756,7 @@
         <v>116</v>
       </c>
       <c r="B12" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="E12" s="5">
         <f>E4+E5</f>
@@ -4692,7 +4767,7 @@
         <v>117</v>
       </c>
       <c r="B13" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="E13" s="5">
         <f>E4+E6</f>
@@ -4703,7 +4778,7 @@
         <v>118</v>
       </c>
       <c r="B14" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="E14" s="5">
         <f>E8+E7</f>
@@ -4711,7 +4786,7 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -4732,28 +4807,28 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B4" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="C4" s="4">
         <f>12*Server!E4</f>
@@ -4761,10 +4836,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="B5" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="C5" s="4">
         <f>5*(Server!E5+Software!C15)</f>
@@ -4772,10 +4847,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="B6" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="C6" s="4">
         <f>7*(Server!E6+Software!D15)</f>
@@ -4783,10 +4858,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B7" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="C7" s="4">
         <v>0</v>
@@ -4794,10 +4869,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="30" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="C8" s="31">
         <f>SUM(C4:C7)</f>
@@ -4805,10 +4880,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B9" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="C9" s="4">
         <f>C8*Asumsi!$C$19</f>
@@ -4816,10 +4891,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="32" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="C10" s="33">
         <f>C8+C9</f>
@@ -4827,21 +4902,21 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B11" s="34" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="C11" s="35" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B12" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="C12" s="4">
         <f>C11-C10</f>
@@ -4849,17 +4924,17 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="B15" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="C15" s="4">
         <f>3600*Asumsi!$C$4</f>
@@ -4867,10 +4942,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="B16" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="C16" s="4">
         <f>12000*Asumsi!$C$4</f>
@@ -4878,10 +4953,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B17" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="C17" s="9">
         <f>C10/C15</f>
@@ -4889,10 +4964,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B18" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="C18" s="9">
         <f>C10/C16</f>
@@ -4900,22 +4975,22 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B23" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C23" s="4">
         <f>12*Server!E4+3*(Server!E5+Software!C15)+9*(Server!E6+Software!D15)</f>
@@ -4923,10 +4998,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B24" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="C24" s="4">
         <f>C23*Asumsi!$C$19</f>
@@ -4934,10 +5009,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="C25" s="5">
         <f>C23+C24</f>
@@ -4945,10 +5020,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B26" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="C26" s="4">
         <f>C11-C25</f>
@@ -4972,7 +5047,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -4980,77 +5055,77 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="B4" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="C4" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D4" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="B5" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="C5" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D5" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="B6" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="C6" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="D6" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="B7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="C7" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="D7" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="18"/>
@@ -5058,7 +5133,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -5066,27 +5141,27 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>
@@ -5108,7 +5183,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -5116,91 +5191,91 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="B4" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C4" s="28">
         <v>150000000</v>
       </c>
       <c r="D4" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="B5" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="C5" s="28">
         <v>40000000</v>
       </c>
       <c r="D5" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="C6" s="28">
         <v>20000000</v>
       </c>
       <c r="D6" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="B7" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="C7" s="28">
         <v>20000000</v>
       </c>
       <c r="D7" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C8" s="5">
         <f>SUM(C4:C7)</f>
       </c>
       <c r="D8" s="18" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="B9" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="C9" s="36">
         <v>4</v>
@@ -5208,10 +5283,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B10" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="C10" s="4">
         <f>C8/(C9*12)</f>
@@ -5219,52 +5294,52 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="B13" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="C13" s="28">
         <v>4500000</v>
       </c>
       <c r="D13" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="B14" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="C14" s="28">
         <v>6500000</v>
       </c>
       <c r="D14" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="B15" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="C15" s="28">
         <v>500000</v>
@@ -5272,21 +5347,21 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C16" s="5">
         <f>SUM(C13:C15)</f>
       </c>
       <c r="D16" s="18" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -5294,24 +5369,24 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B19" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="C19" s="4">
         <f>C16+C10</f>
       </c>
       <c r="D19" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="B20" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="C20" s="4">
         <f>Ringkasan!E7</f>
@@ -5319,10 +5394,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="B21" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="C21" s="4">
         <f>C20-C19</f>
@@ -5330,10 +5405,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="B22" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="C22">
         <f>IF(C23-C19&gt;0,C8/(C23-C19),"—")</f>
@@ -5341,21 +5416,21 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="B23" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="C23" s="28">
         <v>25000000</v>
       </c>
       <c r="D23" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -5366,91 +5441,91 @@
         <v>3</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="B27" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="C27" s="4">
         <f>Anggaran12Bln!C11</f>
       </c>
       <c r="D27" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="B28" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="C28" s="4">
         <f>(5*Ringkasan!E6+7*Ringkasan!E7)*(1+Asumsi!$C$19)</f>
       </c>
       <c r="D28" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="B29" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C29" s="4">
-        <f>(8*Ringkasan!E7+C8+4*(C16+SUM(Software!E22:E24)))*(1+Asumsi!$C$19)</f>
+        <f>(8*Ringkasan!E7+C8+4*(C16+SUM(Software!E22:E25)))*(1+Asumsi!$C$19)</f>
       </c>
       <c r="D29" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="C30" s="8">
         <f>SUM(C27:C29)</f>
       </c>
       <c r="D30" s="7" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="B31" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="C31" s="4">
-        <f>(C16+C10+SUM(Software!E22:E24))*12</f>
+        <f>(C16+C10+SUM(Software!E22:E25))*12</f>
       </c>
       <c r="D31" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="B32" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="C32" s="4">
         <f>(3600+12000+36000)*Asumsi!$C$4</f>
@@ -5458,10 +5533,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="B33" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="C33" s="9">
         <f>C30/C32</f>

</xml_diff>